<commit_message>
Links to spreadsheet of ward level IMD summaries
</commit_message>
<xml_diff>
--- a/imd-ward-sheff.xlsx
+++ b/imd-ward-sheff.xlsx
@@ -1,125 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="25726"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sccextranet-my.sharepoint.com/personal/laurie_platt_sheffield_gov_uk/Documents/Repo/imd-ward-sheff/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_4E78FDCE8F79A8D366075C52F3867A755F09D550" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86C7D4FD-3EED-4BFE-8696-175E72C81748}"/>
   <bookViews>
-    <workbookView xWindow="372" yWindow="-108" windowWidth="22776" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
-  <si>
-    <t>ward_name</t>
-  </si>
-  <si>
-    <t>imd_avg_rank</t>
-  </si>
-  <si>
-    <t>sheff_imd_rank</t>
-  </si>
-  <si>
-    <t>Burngreave</t>
-  </si>
-  <si>
-    <t>Firth Park</t>
-  </si>
-  <si>
-    <t>Southey</t>
-  </si>
-  <si>
-    <t>Manor Castle</t>
-  </si>
-  <si>
-    <t>Shiregreen and Brightside</t>
-  </si>
-  <si>
-    <t>Darnall</t>
-  </si>
-  <si>
-    <t>Park and Arbourthorne</t>
-  </si>
-  <si>
-    <t>Gleadless Valley</t>
-  </si>
-  <si>
-    <t>Richmond</t>
-  </si>
-  <si>
-    <t>Woodhouse</t>
-  </si>
-  <si>
-    <t>Beauchief and Greenhill</t>
-  </si>
-  <si>
-    <t>City</t>
-  </si>
-  <si>
-    <t>Birley</t>
-  </si>
-  <si>
-    <t>Nether Edge and Sharrow</t>
-  </si>
-  <si>
-    <t>Walkley</t>
-  </si>
-  <si>
-    <t>Hillsborough</t>
-  </si>
-  <si>
-    <t>East Ecclesfield</t>
-  </si>
-  <si>
-    <t>Stocksbridge and Upper Don</t>
-  </si>
-  <si>
-    <t>Mosborough</t>
-  </si>
-  <si>
-    <t>Beighton</t>
-  </si>
-  <si>
-    <t>West Ecclesfield</t>
-  </si>
-  <si>
-    <t>Stannington</t>
-  </si>
-  <si>
-    <t>Graves Park</t>
-  </si>
-  <si>
-    <t>Broomhill and Sharrow Vale</t>
-  </si>
-  <si>
-    <t>Dore and Totley</t>
-  </si>
-  <si>
-    <t>Crookes and Crosspool</t>
-  </si>
-  <si>
-    <t>Fulwood</t>
-  </si>
-  <si>
-    <t>Ecclesall</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -167,14 +63,6 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -221,7 +109,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -253,27 +141,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -305,24 +175,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -498,29 +350,32 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C29"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="24.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>3</v>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ward_name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>imd_avg_rank</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>sheff_imd_rank</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Burngreave</t>
+        </is>
       </c>
       <c r="B2">
         <v>2253.5</v>
@@ -529,20 +384,24 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>4</v>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Firth Park</t>
+        </is>
       </c>
       <c r="B3">
-        <v>2349.1999999999998</v>
+        <v>2349.2</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>5</v>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Southey</t>
+        </is>
       </c>
       <c r="B4">
         <v>3641.7</v>
@@ -551,9 +410,11 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>6</v>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Manor Castle</t>
+        </is>
       </c>
       <c r="B5">
         <v>3940.1</v>
@@ -562,20 +423,24 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>7</v>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Shiregreen and Brightside</t>
+        </is>
       </c>
       <c r="B6">
-        <v>4886.8999999999996</v>
+        <v>4886.9</v>
       </c>
       <c r="C6">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>8</v>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Darnall</t>
+        </is>
       </c>
       <c r="B7">
         <v>5084.8</v>
@@ -584,9 +449,11 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>9</v>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Park and Arbourthorne</t>
+        </is>
       </c>
       <c r="B8">
         <v>6040.9</v>
@@ -595,9 +462,11 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>10</v>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Gleadless Valley</t>
+        </is>
       </c>
       <c r="B9">
         <v>8345.5</v>
@@ -606,20 +475,24 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>11</v>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
       </c>
       <c r="B10">
-        <v>10028.799999999999</v>
+        <v>10028.8</v>
       </c>
       <c r="C10">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>12</v>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Woodhouse</t>
+        </is>
       </c>
       <c r="B11">
         <v>10513.3</v>
@@ -628,9 +501,11 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>13</v>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Beauchief and Greenhill</t>
+        </is>
       </c>
       <c r="B12">
         <v>12331</v>
@@ -639,9 +514,11 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>14</v>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
       </c>
       <c r="B13">
         <v>13285.7</v>
@@ -650,9 +527,11 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>15</v>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Birley</t>
+        </is>
       </c>
       <c r="B14">
         <v>13366.4</v>
@@ -661,9 +540,11 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>16</v>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Nether Edge and Sharrow</t>
+        </is>
       </c>
       <c r="B15">
         <v>13737.7</v>
@@ -672,9 +553,11 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>17</v>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Walkley</t>
+        </is>
       </c>
       <c r="B16">
         <v>14427.4</v>
@@ -683,9 +566,11 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>18</v>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Hillsborough</t>
+        </is>
       </c>
       <c r="B17">
         <v>15745.1</v>
@@ -694,64 +579,76 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>19</v>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>East Ecclesfield</t>
+        </is>
       </c>
       <c r="B18">
-        <v>16661.400000000001</v>
+        <v>16661.4</v>
       </c>
       <c r="C18">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>20</v>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Stocksbridge and Upper Don</t>
+        </is>
       </c>
       <c r="B19">
-        <v>16813.599999999999</v>
+        <v>16813.6</v>
       </c>
       <c r="C19">
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>21</v>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Mosborough</t>
+        </is>
       </c>
       <c r="B20">
-        <v>16925.400000000001</v>
+        <v>16925.4</v>
       </c>
       <c r="C20">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>22</v>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Beighton</t>
+        </is>
       </c>
       <c r="B21">
-        <v>16972.099999999999</v>
+        <v>16972.1</v>
       </c>
       <c r="C21">
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>23</v>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>West Ecclesfield</t>
+        </is>
       </c>
       <c r="B22">
-        <v>18729.099999999999</v>
+        <v>18729.1</v>
       </c>
       <c r="C22">
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>24</v>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Stannington</t>
+        </is>
       </c>
       <c r="B23">
         <v>20632</v>
@@ -760,9 +657,11 @@
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>25</v>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Graves Park</t>
+        </is>
       </c>
       <c r="B24">
         <v>21100.6</v>
@@ -771,20 +670,24 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>26</v>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Broomhill and Sharrow Vale</t>
+        </is>
       </c>
       <c r="B25">
-        <v>21934.799999999999</v>
+        <v>21934.8</v>
       </c>
       <c r="C25">
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>27</v>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Dore and Totley</t>
+        </is>
       </c>
       <c r="B26">
         <v>27180.3</v>
@@ -793,9 +696,11 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>28</v>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Crookes and Crosspool</t>
+        </is>
       </c>
       <c r="B27">
         <v>28078.9</v>
@@ -804,9 +709,11 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>29</v>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Fulwood</t>
+        </is>
       </c>
       <c r="B28">
         <v>29822.9</v>
@@ -815,9 +722,11 @@
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>30</v>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Ecclesall</t>
+        </is>
       </c>
       <c r="B29">
         <v>30618.1</v>

</xml_diff>